<commit_message>
feat: complete SalesGenie AI implementation with conversation intelligence, AI sales strategy matrix, and CRM integration
</commit_message>
<xml_diff>
--- a/SalesGenie DATA/Github Repository.xlsx
+++ b/SalesGenie DATA/Github Repository.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
   <si>
     <t>AI Sales Intelligence Platform Group -2</t>
   </si>
@@ -110,6 +110,9 @@
     <t>arshadkalimalla89@gmail.com</t>
   </si>
   <si>
+    <t>https://github.com/Arshad2k57815/ElectronicsSalesDashboard</t>
+  </si>
+  <si>
     <t>Kandula Varun</t>
   </si>
   <si>
@@ -191,13 +194,13 @@
     <t>tgas10476@gmail.com</t>
   </si>
   <si>
+    <t>https://github.com/shubh152205/AnimeGenie_ShubhamSharma</t>
+  </si>
+  <si>
     <t>Shubham Sharma</t>
   </si>
   <si>
     <t>shubham8423286406@gmail.com</t>
-  </si>
-  <si>
-    <t>https://github.com/shubh152205/AnimeGenie_ShubhamSharma</t>
   </si>
   <si>
     <t>Srinivas B N</t>
@@ -234,7 +237,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -280,6 +283,12 @@
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.0"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
@@ -374,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -400,10 +409,10 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -411,8 +420,11 @@
     <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="13" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -757,174 +769,175 @@
       <c r="B15" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="7"/>
+      <c r="C15" s="10" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C20" s="7"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="10" t="s">
         <v>48</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" s="11" t="s">
         <v>51</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="C24" s="12" t="s">
         <v>54</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25" s="7"/>
+        <v>57</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C28" s="13" t="s">
         <v>65</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B29" s="15" t="s">
+      <c r="A29" s="15" t="s">
         <v>67</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>68</v>
       </c>
       <c r="C29" s="7"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C30" s="7"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
+      <c r="A31" s="17"/>
+      <c r="B31" s="17"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="16"/>
-      <c r="B32" s="16"/>
+      <c r="A32" s="17"/>
+      <c r="B32" s="17"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="16"/>
-      <c r="B33" s="16"/>
+      <c r="A33" s="17"/>
+      <c r="B33" s="17"/>
     </row>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -1910,36 +1923,37 @@
     <hyperlink r:id="rId13" ref="B13"/>
     <hyperlink r:id="rId14" ref="B14"/>
     <hyperlink r:id="rId15" ref="B15"/>
-    <hyperlink r:id="rId16" ref="B16"/>
-    <hyperlink r:id="rId17" ref="C16"/>
-    <hyperlink r:id="rId18" ref="B17"/>
-    <hyperlink r:id="rId19" ref="C17"/>
-    <hyperlink r:id="rId20" ref="B18"/>
-    <hyperlink r:id="rId21" ref="C18"/>
-    <hyperlink r:id="rId22" ref="B19"/>
-    <hyperlink r:id="rId23" ref="B20"/>
-    <hyperlink r:id="rId24" ref="B21"/>
-    <hyperlink r:id="rId25" ref="C21"/>
-    <hyperlink r:id="rId26" ref="B22"/>
-    <hyperlink r:id="rId27" ref="C22"/>
-    <hyperlink r:id="rId28" ref="B23"/>
-    <hyperlink r:id="rId29" ref="C23"/>
-    <hyperlink r:id="rId30" ref="B24"/>
-    <hyperlink r:id="rId31" ref="C24"/>
-    <hyperlink r:id="rId32" ref="B25"/>
-    <hyperlink r:id="rId33" ref="B26"/>
-    <hyperlink r:id="rId34" ref="C26"/>
-    <hyperlink r:id="rId35" ref="B27"/>
-    <hyperlink r:id="rId36" ref="C27"/>
-    <hyperlink r:id="rId37" ref="B28"/>
-    <hyperlink r:id="rId38" ref="C28"/>
-    <hyperlink r:id="rId39" ref="B29"/>
-    <hyperlink r:id="rId40" ref="B30"/>
+    <hyperlink r:id="rId16" ref="C15"/>
+    <hyperlink r:id="rId17" ref="B16"/>
+    <hyperlink r:id="rId18" ref="C16"/>
+    <hyperlink r:id="rId19" ref="B17"/>
+    <hyperlink r:id="rId20" ref="C17"/>
+    <hyperlink r:id="rId21" ref="B18"/>
+    <hyperlink r:id="rId22" ref="C18"/>
+    <hyperlink r:id="rId23" ref="B19"/>
+    <hyperlink r:id="rId24" ref="B20"/>
+    <hyperlink r:id="rId25" ref="B21"/>
+    <hyperlink r:id="rId26" ref="C21"/>
+    <hyperlink r:id="rId27" ref="B22"/>
+    <hyperlink r:id="rId28" ref="C22"/>
+    <hyperlink r:id="rId29" ref="B23"/>
+    <hyperlink r:id="rId30" ref="C23"/>
+    <hyperlink r:id="rId31" ref="B24"/>
+    <hyperlink r:id="rId32" ref="C24"/>
+    <hyperlink r:id="rId33" ref="B25"/>
+    <hyperlink r:id="rId34" ref="C25"/>
+    <hyperlink r:id="rId35" ref="B26"/>
+    <hyperlink r:id="rId36" ref="B27"/>
+    <hyperlink r:id="rId37" ref="C27"/>
+    <hyperlink r:id="rId38" ref="B28"/>
+    <hyperlink r:id="rId39" ref="C28"/>
+    <hyperlink r:id="rId40" ref="B29"/>
+    <hyperlink r:id="rId41" ref="B30"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait"/>
-  <drawing r:id="rId41"/>
+  <drawing r:id="rId42"/>
 </worksheet>
 </file>
 

</xml_diff>